<commit_message>
Expand plans, progress, personas, and sound controls
</commit_message>
<xml_diff>
--- a/media not in app/Plans.xlsx
+++ b/media not in app/Plans.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="53">
   <si>
     <t>Cope plan</t>
   </si>
@@ -162,25 +162,19 @@
     <t>Acceptance</t>
   </si>
   <si>
-    <t>Let it go</t>
-  </si>
-  <si>
     <t>Forgiveness</t>
   </si>
   <si>
-    <t>Is there someone you can forgive now? Or someone you feel ready to ask for forgiveness?</t>
-  </si>
-  <si>
-    <t>Is there some issue you need to let go of?</t>
-  </si>
-  <si>
     <t>In the evening, meditate on the next steps you can take to further vanquish your anxiety</t>
   </si>
   <si>
-    <t>Is there something you've been struggling to accept?</t>
-  </si>
-  <si>
-    <t>Relect on the insights from the Understand phase</t>
+    <t>Reflect on the insights from the Understand phase</t>
+  </si>
+  <si>
+    <t>forgive what needs to be forgiven</t>
+  </si>
+  <si>
+    <t>Let go of what has been worrying you</t>
   </si>
 </sst>
 </file>
@@ -268,14 +262,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,19 +641,19 @@
       <c r="A10" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="7"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="7"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -684,7 +678,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>28</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -695,7 +689,7 @@
       <c r="A15" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="6" t="s">
@@ -706,7 +700,7 @@
       <c r="A16" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
       <c r="E16" s="6" t="s">
@@ -714,7 +708,7 @@
       </c>
     </row>
     <row r="17" spans="4:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E17" s="6" t="s">
@@ -791,10 +785,10 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="7"/>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C13" s="3" t="s">
@@ -805,7 +799,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>39</v>
       </c>
       <c r="D14" s="6" t="s">
@@ -813,7 +807,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -821,7 +815,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -829,7 +823,7 @@
       </c>
     </row>
     <row r="17" spans="3:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -837,7 +831,7 @@
       </c>
     </row>
     <row r="18" spans="3:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>37</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -854,7 +848,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.28515625" customWidth="1"/>
@@ -912,10 +906,10 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="7"/>
+      <c r="D10" s="9"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C11" s="3" t="s">
@@ -925,44 +919,41 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="C12" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C14" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="C14" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="C15" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="C16" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="6" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
@@ -977,11 +968,6 @@
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>